<commit_message>
Fill indexed pages for lefooding.com
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CqzDhzdNSwoc2HngfH4ZQ9
</commit_message>
<xml_diff>
--- a/Analyse_popularite_sites_Uber_Eats.xlsx
+++ b/Analyse_popularite_sites_Uber_Eats.xlsx
@@ -510,7 +510,11 @@
           <t>Guide des restaurants</t>
         </is>
       </c>
-      <c r="C4" s="3" t="n"/>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Environ 42 100</t>
+        </is>
+      </c>
       <c r="D4" s="3" t="n"/>
       <c r="E4" s="3" t="n"/>
     </row>

</xml_diff>

<commit_message>
Fill domain age and authority for lefooding.com
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CqzDhzdNSwoc2HngfH4ZQ9
</commit_message>
<xml_diff>
--- a/Analyse_popularite_sites_Uber_Eats.xlsx
+++ b/Analyse_popularite_sites_Uber_Eats.xlsx
@@ -515,8 +515,16 @@
           <t>Environ 42 100</t>
         </is>
       </c>
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="3" t="n"/>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Créé en 2001 (25 ans)</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>63/100</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Fill indexed pages for 750g.com and thefork.fr
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CqzDhzdNSwoc2HngfH4ZQ9
</commit_message>
<xml_diff>
--- a/Analyse_popularite_sites_Uber_Eats.xlsx
+++ b/Analyse_popularite_sites_Uber_Eats.xlsx
@@ -552,7 +552,11 @@
           <t>Recettes de cuisine</t>
         </is>
       </c>
-      <c r="C6" s="3" t="n"/>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Environ 132 000</t>
+        </is>
+      </c>
       <c r="D6" s="3" t="n"/>
       <c r="E6" s="3" t="n"/>
     </row>
@@ -567,7 +571,11 @@
           <t>Réservation de restaurants</t>
         </is>
       </c>
-      <c r="C7" s="4" t="n"/>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Environ 321 000</t>
+        </is>
+      </c>
       <c r="D7" s="4" t="n"/>
       <c r="E7" s="4" t="n"/>
     </row>

</xml_diff>

<commit_message>
Add Marmiton and Moz scores to netlinking PDF and Excel
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CqzDhzdNSwoc2HngfH4ZQ9
</commit_message>
<xml_diff>
--- a/Analyse_popularite_sites_Uber_Eats.xlsx
+++ b/Analyse_popularite_sites_Uber_Eats.xlsx
@@ -537,9 +537,21 @@
           <t>Recettes de cuisine</t>
         </is>
       </c>
-      <c r="C5" s="4" t="n"/>
-      <c r="D5" s="4" t="n"/>
-      <c r="E5" s="4" t="n"/>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Environ 356 000</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Créé en 2002 (24 ans)</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>83/100</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -558,7 +570,11 @@
         </is>
       </c>
       <c r="D6" s="3" t="n"/>
-      <c r="E6" s="3" t="n"/>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>82/100</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -577,7 +593,11 @@
         </is>
       </c>
       <c r="D7" s="4" t="n"/>
-      <c r="E7" s="4" t="n"/>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>65/100</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add creation dates for 750g and thefork
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CqzDhzdNSwoc2HngfH4ZQ9
</commit_message>
<xml_diff>
--- a/Analyse_popularite_sites_Uber_Eats.xlsx
+++ b/Analyse_popularite_sites_Uber_Eats.xlsx
@@ -569,7 +569,11 @@
           <t>Environ 132 000</t>
         </is>
       </c>
-      <c r="D6" s="3" t="n"/>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Créé en 2025 (1 an)</t>
+        </is>
+      </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
           <t>82/100</t>
@@ -592,7 +596,11 @@
           <t>Environ 321 000</t>
         </is>
       </c>
-      <c r="D7" s="4" t="n"/>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Créé en 2014 (12 ans)</t>
+        </is>
+      </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
           <t>65/100</t>

</xml_diff>